<commit_message>
refactor: simplify login test suite, remove AI boilerplate and optimize page objects
</commit_message>
<xml_diff>
--- a/test_data/login_test_cases.xlsx
+++ b/test_data/login_test_cases.xlsx
@@ -887,7 +887,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-08-12 16:11:22</t>
+          <t>2026-08-13 19:55:51</t>
         </is>
       </c>
     </row>
@@ -946,7 +946,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-08-12 16:11:25</t>
+          <t>2026-08-13 19:55:54</t>
         </is>
       </c>
     </row>
@@ -1119,19 +1119,20 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-08-12 16:12:02</t>
+          <t>2026-08-13 19:56:22</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>tests\test_login.py:204: in test_2fa_back_to_login_link_TC_LOGIN_005
-    login_pg.navigate()
-pages\login_page.py:64: in navigate
-    self.page.goto(url, wait_until="networkidle", timeout=30_000)
-..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwright\sync_api\_generated.py:9875: in goto
+          <t>tests\test_login.py:101: in test_2fa_back_to_login_TC_LOGIN_005
+    lp.login(creds["employee_id"], creds["password"])
+pages\login_page.py:66: in login
+    self.enter_employee_id(emp_id)
+pages\login_page.py:54: in enter_employee_id
+    self.employee_id_input.fill(str(emp_id))
+..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwright\sync_api\_generated.py:18242: in fill
     self._sync(
-..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwright\_impl\_page.py:560: in goto
-    return await self._main_frame.goto(**locals_to_params(locals()))</t>
+..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwright\_impl\_locator</t>
         </is>
       </c>
     </row>
@@ -1183,24 +1184,25 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="K11" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-08-12 16:12:17</t>
+          <t>2026-08-13 19:56:41</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>tests\test_login.py:267: in test_logout_flow_TC_LOGIN_006
-    assert login_pg2.is_employee_id_field_visible(), (
-E   AssertionError: Not returned to login page after logout. URL: https://swarajya-stg.corecotechnologies.com/logout
-E   assert False
-E    +  where False = is_employee_id_field_visible()
-E    +    where is_employee_id_field_visible = &lt;pages.login_page.LoginPage object at 0x00000224B78475C0&gt;.is_employee_id_field_visible</t>
+          <t>self = &lt;tests.test_login.TestLoginFlows object at 0x0000020CFB427610&gt;
+page = &lt;Page url='https://swarajya-stg.corecotechnologies.com/'&gt;
+base_url = 'https://swarajya-stg.corecotechnologies.com'
+employee_credentials = {'role': 'Employee', 'employee_id': '332', 'password': 'test@1234', 'auth_code': '111111', ...}
+    def test_logout_TC_LOGIN_006(self, page, base_url, employee_credentials):
+        """After full login, logging out should land back on the sign-in page."""
+        creds = employee_cre</t>
         </is>
       </c>
     </row>
@@ -1258,7 +1260,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-08-12 16:11:30</t>
+          <t>2026-08-13 19:55:58</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1917,7 +1919,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-08-12 16:12:35</t>
+          <t>2026-08-13 19:57:01</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1980,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-08-12 16:12:40</t>
+          <t>2026-08-13 19:57:06</t>
         </is>
       </c>
     </row>
@@ -2039,7 +2041,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-08-12 16:12:45</t>
+          <t>2026-08-13 19:57:11</t>
         </is>
       </c>
     </row>
@@ -2100,7 +2102,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-08-12 16:12:50</t>
+          <t>2026-08-13 19:57:15</t>
         </is>
       </c>
     </row>
@@ -2161,7 +2163,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-08-12 16:13:01</t>
+          <t>2026-08-13 19:57:21</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -2220,14 +2222,14 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="K15" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K15" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-08-12 16:13:14</t>
+          <t>2026-08-13 19:57:27</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2300,7 +2302,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-08-12 16:13:20</t>
+          <t>2026-08-13 19:57:33</t>
         </is>
       </c>
     </row>
@@ -2361,7 +2363,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-08-12 16:13:27</t>
+          <t>2026-08-13 19:57:37</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2427,19 +2429,21 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-08-12 16:13:41</t>
+          <t>2026-08-13 19:51:44</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>tests\test_login.py:543: in test_xss_injection_TC_LOGIN_017
-    login_page.enter_employee_id("&lt;script&gt;alert(1)&lt;/script&gt;")
-pages\login_page.py:73: in enter_employee_id
-    self.employee_id_input.fill(str(employee_id))
-..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwright\sync_api\_generated.py:18242: in fill
-    self._sync(
-..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwright\_impl\_locator.py:219: in fill
-    return await self._frame.fill(self._se</t>
+          <t xml:space="preserve">self = &lt;tests.test_login.TestNegativeLoginGeneral object at 0x0000020CFB433B50&gt;
+page = &lt;Page url='https://swarajya-stg.corecotechnologies.com/'&gt;
+base_url = 'https://swarajya-stg.corecotechnologies.com'
+    @pytest.mark.security
+    def test_xss_injection_TC_LOGIN_017(self, page, base_url):
+        """XSS payload must not execute or bypass auth."""
+        # dismiss any JS dialogs the XSS might trigger
+        page.on("dialog", lambda d: d.dismiss())
+        lp = LoginPage(page, base_url)
+ </t>
         </is>
       </c>
     </row>
@@ -2500,19 +2504,21 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-08-12 16:13:56</t>
+          <t>2026-08-13 19:51:57</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>tests\test_login.py:565: in test_employee_id_exceeding_length_TC_LOGIN_018
-    login_page.enter_employee_id(long_id)
-pages\login_page.py:73: in enter_employee_id
-    self.employee_id_input.fill(str(employee_id))
-..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwright\sync_api\_generated.py:18242: in fill
-    self._sync(
-..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwright\_impl\_locator.py:219: in fill
-    return await self._frame.fill(self._selecto</t>
+          <t xml:space="preserve">self = &lt;tests.test_login.TestNegativeLoginGeneral object at 0x0000020CFB4A4B90&gt;
+page = &lt;Page url='https://swarajya-stg.corecotechnologies.com/'&gt;
+base_url = 'https://swarajya-stg.corecotechnologies.com'
+    def test_long_employee_id_TC_LOGIN_018(self, page, base_url):
+        """ID exceeding 256 chars — should be handled gracefully."""
+        lp = LoginPage(page, base_url)
+        lp.navigate()
+&gt;       lp.enter_employee_id("A" * 300)
+swarajya-automation\tests\test_login.py:281: 
+_ _ _ _ _ _ _ </t>
         </is>
       </c>
     </row>
@@ -2573,19 +2579,18 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-08-12 16:14:08</t>
+          <t>2026-08-13 19:52:09</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>tests\test_login.py:589: in test_password_exceeding_length_TC_LOGIN_019
-    login_page.enter_employee_id(creds["employee_id"])
-pages\login_page.py:73: in enter_employee_id
-    self.employee_id_input.fill(str(employee_id))
-..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwright\sync_api\_generated.py:18242: in fill
-    self._sync(
-..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwright\_impl\_locator.py:219: in fill
-    return await self._frame.fill(sel</t>
+          <t>self = &lt;tests.test_login.TestNegativeLoginGeneral object at 0x0000020CFB4A6120&gt;
+page = &lt;Page url='https://swarajya-stg.corecotechnologies.com/'&gt;
+base_url = 'https://swarajya-stg.corecotechnologies.com'
+employee_credentials = {'role': 'Employee', 'employee_id': '332', 'password': 'test@1234', 'auth_code': '111111', ...}
+    def test_long_password_TC_LOGIN_019(self, page, base_url, employee_credentials):
+        """Password exceeding 256 chars — should be handled gracefully."""
+        lp = Login</t>
         </is>
       </c>
     </row>
@@ -2639,14 +2644,14 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="K21" s="8" t="inlineStr">
-        <is>
-          <t>SKIPPED</t>
+      <c r="K21" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-08-12 16:16:01</t>
+          <t>2026-08-13 19:54:02</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2712,19 +2717,18 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-08-12 16:14:21</t>
+          <t>2026-08-13 19:52:21</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>tests\test_login.py:615: in test_case_sensitive_password_TC_LOGIN_021
-    login_page.enter_employee_id(creds["employee_id"])
-pages\login_page.py:73: in enter_employee_id
-    self.employee_id_input.fill(str(employee_id))
-..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwright\sync_api\_generated.py:18242: in fill
-    self._sync(
-..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwright\_impl\_locator.py:219: in fill
-    return await self._frame.fill(self.</t>
+          <t>self = &lt;tests.test_login.TestNegativeLoginGeneral object at 0x0000020CFB511B70&gt;
+login_page = &lt;pages.login_page.LoginPage object at 0x0000020CFBAA3E70&gt;
+employee_credentials = {'role': 'Employee', 'employee_id': '332', 'password': 'test@1234', 'auth_code': '111111', ...}
+    def test_case_sensitive_password_TC_LOGIN_021(self, login_page, employee_credentials):
+        """Swapped-case password should be rejected."""
+        creds = employee_credentials
+&gt;       login_page.enter_employee_id(creds["e</t>
         </is>
       </c>
     </row>
@@ -2783,20 +2787,18 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-08-12 16:14:34</t>
+          <t>2026-08-13 19:52:29</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>tests\test_login.py:649: in test_incorrect_2fa_code_TC_LOGIN_022
-    login_pg.login(creds["employee_id"], creds["password"])
-pages\login_page.py:94: in login
-    self.enter_employee_id(employee_id)
-pages\login_page.py:73: in enter_employee_id
-    self.employee_id_input.fill(str(employee_id))
-..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwright\sync_api\_generated.py:18242: in fill
-    self._sync(
-..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwrig</t>
+          <t>self = &lt;tests.test_login.TestNegative2FA object at 0x0000020CFB427D90&gt;
+page = &lt;Page url='https://swarajya-stg.corecotechnologies.com/default'&gt;
+base_url = 'https://swarajya-stg.corecotechnologies.com'
+employee_credentials = {'role': 'Employee', 'employee_id': '332', 'password': 'test@1234', 'auth_code': '111111', ...}
+    def test_wrong_2fa_code_TC_LOGIN_022(self, page, base_url, employee_credentials):
+        """Incorrect 2FA code should not proceed to dashboard."""
+        tfa = self._login_an</t>
         </is>
       </c>
     </row>
@@ -2855,7 +2857,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-08-12 16:14:40</t>
+          <t>2026-08-13 19:52:36</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2921,14 +2923,14 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="K25" s="8" t="inlineStr">
-        <is>
-          <t>SKIPPED</t>
+      <c r="K25" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-08-12 16:16:01</t>
+          <t>2026-08-13 19:54:05</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2987,14 +2989,14 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="K26" s="8" t="inlineStr">
-        <is>
-          <t>SKIPPED</t>
+      <c r="K26" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-08-12 16:16:01</t>
+          <t>2026-08-13 19:54:09</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3051,25 +3053,26 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="K27" s="7" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="K27" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-08-12 16:14:44</t>
+          <t>2026-08-13 19:52:53</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t xml:space="preserve">tests\test_login.py:712: in test_direct_2fa_url_access_TC_LOGIN_026
-    assert not tfa_pg.is_on_tfa_page() or "/fake-token" not in current_url, (
-E   AssertionError: Direct 2FA access should be denied. URL: https://swarajya-stg.corecotechnologies.com/tfa-authcode/fake-token-12345
-E   assert (not True or '/fake-token' not in 'https://swa...-token-12345'
+          <t>tests\test_login.py:334: in test_direct_2fa_url_TC_LOGIN_026
+    assert not tfa.is_on_tfa_page() or "/fake-token" not in page.url
+E   AssertionError: assert (not True or '/fake-token' not in 'https://swarajya-stg.corecotechnologies.com/tfa-authcode/fake-token-12345'
 E    +  where True = is_on_tfa_page()
-E    +    where is_on_tfa_page = &lt;pages.tfa_page.TfaPage object at 0x00000224B7942CF0&gt;.is_on_tfa_page
-E    </t>
+E    +    where is_on_tfa_page = &lt;pages.tfa_page.TfaPage object at 0x000001C25D9F5BF0&gt;.is_on_tfa_page
+E     
+E     '/fake-token' is contained here:
+E       https://swarajya-stg.corecotechnologies</t>
         </is>
       </c>
     </row>
@@ -3128,416 +3131,427 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-08-12 16:15:09</t>
+          <t>2026-08-13 19:51:54</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>tests\test_login.py:736: in test_repeated_failed_2fa_attempts_TC_LOGIN_027
-    tfa_pg.enter_auth_code(f"00000{attempt}")
-pages\tfa_page.py:80: in enter_auth_code
-    self.auth_code_input.fill(str(code))
+          <t>tests\test_login.py:362: in test_repeated_wrong_2fa_TC_LOGIN_027
+    tfa = self._login_and_reach_2fa(page, base_url, employee_credentials)
+          ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
+tests\test_login.py:323: in _login_and_reach_2fa
+    lp.login(creds["employee_id"], creds["password"])
+pages\login_page.py:66: in login
+    self.enter_employee_id(emp_id)
+pages\login_page.py:54: in enter_employee_id
+    self.employee_id_input.fill(str(emp_id))
+..\..\..\AppData\Local\Pro</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="62" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_028</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Verify a failed login attempt does not grant application access</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Login page is accessible</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>1. Enter invalid credentials
+2. Click Sign In
+3. Attempt to open an authenticated page</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>Invalid Employee ID and password</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>The user is not authenticated and is not granted access to protected pages</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr"/>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>To Be Automated</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="K29" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-08-13 19:53:15</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>tests\test_login.py:390: in test_failed_login_no_access_TC_LOGIN_028
+    lp.login("INVALID_USER", "Invalid@123")
+pages\login_page.py:66: in login
+    self.enter_employee_id(emp_id)
+pages\login_page.py:54: in enter_employee_id
+    self.employee_id_input.fill(str(emp_id))
+..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwright\sync_api\_generated.py:18242: in fill
+    self._sync(
+..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwright\_impl\_locator.py:2</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="62" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_029</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Verify an unauthenticated user cannot access the dashboard directly</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>User is logged out</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>1. Open the protected dashboard URL directly without logging in</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Protected dashboard URL</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>The user is redirected to the login page or access is denied</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr"/>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>To Be Automated</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="K30" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-08-13 19:53:19</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>tests\test_login.py:402: in test_unauthenticated_dashboard_TC_LOGIN_029
+    assert lp.is_employee_id_field_visible() or "/default" not in page.url
+E   AssertionError: assert (False or '/default' not in 'https://swarajya-stg.corecotechnologies.com/default'
+E    +  where False = is_employee_id_field_visible()
+E    +    where is_employee_id_field_visible = &lt;pages.login_page.LoginPage object at 0x000001787098D250&gt;.is_employee_id_field_visible
+E     
+E     '/default' is contained here:
+E       https:</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="62" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_030</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Verify an HR user cannot access Admin-only functionality</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Valid HR account exists</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>1. Complete login as HR
+2. Attempt to access Admin-only functionality</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>HR credentials and Admin URL/functionality</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>HR is denied access to Admin-only functionality</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr"/>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>To Be Automated</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="K31" s="8" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-08-13 19:54:09</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Skipped: RBAC not implemented in staging</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="62" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_031</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Verify an Employee-role user cannot access Admin-only functionality</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>Valid Employee account exists</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>1. Complete login as Employee
+2. Attempt to access Admin-only functionality</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Employee credentials and Admin URL/functionality</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>Employee is denied access to Admin-only functionality</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr"/>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>To Be Automated</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="K32" s="8" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-08-13 19:54:09</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>Skipped: RBAC not implemented in staging</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="62" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_032</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Verify a Manager user cannot access Admin-only functionality</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Valid Manager account exists</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>1. Complete login as Manager
+2. Attempt to access Admin-only functionality</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Manager credentials and Admin URL/functionality</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>Manager is denied access to Admin-only functionality</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr"/>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>To Be Automated</t>
+        </is>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="K33" s="8" t="inlineStr">
+        <is>
+          <t>SKIPPED</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>2026-08-13 19:54:09</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>Skipped: RBAC not implemented in staging</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="62" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>TC_LOGIN_033</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Verify application behaviour on repeated failed Sign In attempts</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Login page is accessible</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>1. Enter incorrect credentials repeatedly
+2. Observe the application response</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Invalid credentials, repeated</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>The configured security control (rate limiting, account lockout, CAPTCHA or a warning) is applied</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr"/>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>To Be Automated</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="K34" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-08-13 19:53:40</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>tests\test_login.py:409: in test_repeated_failed_logins_TC_LOGIN_033
+    login_page.enter_employee_id(f"WRONG_{i}")
+pages\login_page.py:54: in enter_employee_id
+    self.employee_id_input.fill(str(emp_id))
 ..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwright\sync_api\_generated.py:18242: in fill
     self._sync(
 ..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwright\_impl\_locator.py:219: in fill
-    return await self._frame.fill(self._selector, strict</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="62" customHeight="1">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>TC_LOGIN_028</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>Verify a failed login attempt does not grant application access</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>Login page is accessible</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>1. Enter invalid credentials
-2. Click Sign In
-3. Attempt to open an authenticated page</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>Invalid Employee ID and password</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>The user is not authenticated and is not granted access to protected pages</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr"/>
-      <c r="I29" s="3" t="inlineStr">
-        <is>
-          <t>To Be Automated</t>
-        </is>
-      </c>
-      <c r="J29" s="3" t="inlineStr">
-        <is>
-          <t>UI</t>
-        </is>
-      </c>
-      <c r="K29" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>2026-08-12 16:15:17</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>tests\test_login.py:769: in test_failed_login_no_access_TC_LOGIN_028
-    login_pg.navigate()
-pages\login_page.py:64: in navigate
-    self.page.goto(url, wait_until="networkidle", timeout=30_000)
-..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwright\sync_api\_generated.py:9875: in goto
-    self._sync(
-..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwright\_impl\_page.py:560: in goto
-    return await self._main_frame.goto(**locals_to_params(locals()))</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="62" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>TC_LOGIN_029</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>Verify an unauthenticated user cannot access the dashboard directly</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>User is logged out</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>1. Open the protected dashboard URL directly without logging in</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>Protected dashboard URL</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t>The user is redirected to the login page or access is denied</t>
-        </is>
-      </c>
-      <c r="H30" s="3" t="inlineStr"/>
-      <c r="I30" s="3" t="inlineStr">
-        <is>
-          <t>To Be Automated</t>
-        </is>
-      </c>
-      <c r="J30" s="3" t="inlineStr">
-        <is>
-          <t>UI</t>
-        </is>
-      </c>
-      <c r="K30" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>2026-08-12 16:15:22</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>tests\test_login.py:793: in test_unauthenticated_dashboard_access_TC_LOGIN_029
-    page.goto(f"{base_url}/default", timeout=15_000)
-..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwright\sync_api\_generated.py:9875: in goto
-    self._sync(
-..\..\..\AppData\Local\Programs\Python\Python313\Lib\site-packages\playwright\_impl\_page.py:560: in goto
-    return await self._main_frame.goto(**locals_to_params(locals()))
-           ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="62" customHeight="1">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>TC_LOGIN_030</t>
-        </is>
-      </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>Verify an HR user cannot access Admin-only functionality</t>
-        </is>
-      </c>
-      <c r="D31" s="4" t="inlineStr">
-        <is>
-          <t>Valid HR account exists</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>1. Complete login as HR
-2. Attempt to access Admin-only functionality</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>HR credentials and Admin URL/functionality</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t>HR is denied access to Admin-only functionality</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr"/>
-      <c r="I31" s="3" t="inlineStr">
-        <is>
-          <t>To Be Automated</t>
-        </is>
-      </c>
-      <c r="J31" s="3" t="inlineStr">
-        <is>
-          <t>UI</t>
-        </is>
-      </c>
-      <c r="K31" s="8" t="inlineStr">
-        <is>
-          <t>SKIPPED</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>2026-08-12 16:16:01</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>Skipped: BLOCKED: RBAC not implemented — no separate HR/Admin accounts</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="62" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>TC_LOGIN_031</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>Verify an Employee-role user cannot access Admin-only functionality</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>Valid Employee account exists</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>1. Complete login as Employee
-2. Attempt to access Admin-only functionality</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>Employee credentials and Admin URL/functionality</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t>Employee is denied access to Admin-only functionality</t>
-        </is>
-      </c>
-      <c r="H32" s="3" t="inlineStr"/>
-      <c r="I32" s="3" t="inlineStr">
-        <is>
-          <t>To Be Automated</t>
-        </is>
-      </c>
-      <c r="J32" s="3" t="inlineStr">
-        <is>
-          <t>UI</t>
-        </is>
-      </c>
-      <c r="K32" s="8" t="inlineStr">
-        <is>
-          <t>SKIPPED</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>2026-08-12 16:16:01</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>Skipped: BLOCKED: RBAC not implemented — no separate Employee/Admin accounts</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="62" customHeight="1">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>TC_LOGIN_032</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>Verify a Manager user cannot access Admin-only functionality</t>
-        </is>
-      </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>Valid Manager account exists</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>1. Complete login as Manager
-2. Attempt to access Admin-only functionality</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>Manager credentials and Admin URL/functionality</t>
-        </is>
-      </c>
-      <c r="G33" s="4" t="inlineStr">
-        <is>
-          <t>Manager is denied access to Admin-only functionality</t>
-        </is>
-      </c>
-      <c r="H33" s="3" t="inlineStr"/>
-      <c r="I33" s="3" t="inlineStr">
-        <is>
-          <t>To Be Automated</t>
-        </is>
-      </c>
-      <c r="J33" s="3" t="inlineStr">
-        <is>
-          <t>UI</t>
-        </is>
-      </c>
-      <c r="K33" s="8" t="inlineStr">
-        <is>
-          <t>SKIPPED</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>2026-08-12 16:16:02</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>Skipped: BLOCKED: RBAC not implemented — no separate Manager/Admin accounts</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="62" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>TC_LOGIN_033</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>General</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>Verify application behaviour on repeated failed Sign In attempts</t>
-        </is>
-      </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>Login page is accessible</t>
-        </is>
-      </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t>1. Enter incorrect credentials repeatedly
-2. Observe the application response</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>Invalid credentials, repeated</t>
-        </is>
-      </c>
-      <c r="G34" s="4" t="inlineStr">
-        <is>
-          <t>The configured security control (rate limiting, account lockout, CAPTCHA or a warning) is applied</t>
-        </is>
-      </c>
-      <c r="H34" s="3" t="inlineStr"/>
-      <c r="I34" s="3" t="inlineStr">
-        <is>
-          <t>To Be Automated</t>
-        </is>
-      </c>
-      <c r="J34" s="3" t="inlineStr">
-        <is>
-          <t>UI</t>
-        </is>
-      </c>
-      <c r="K34" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>2026-08-12 16:15:43</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>Application responded to 5 failed attempts with error messages</t>
+    return await self._frame.fill(self._selector, str</t>
         </is>
       </c>
     </row>
@@ -3590,14 +3604,14 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="K35" s="8" t="inlineStr">
-        <is>
-          <t>SKIPPED</t>
+      <c r="K35" s="6" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-08-12 16:16:02</t>
+          <t>2026-08-13 19:54:15</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -3655,19 +3669,25 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="K36" s="6" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="K36" s="7" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-08-12 16:16:01</t>
+          <t>2026-08-13 19:53:59</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>URL after back button: https://swarajya-stg.corecotechnologies.com/default</t>
+          <t xml:space="preserve">self = &lt;tests.test_login.TestSecurityAndSession object at 0x0000020CFB4DD480&gt;
+page = &lt;Page url='https://swarajya-stg.corecotechnologies.com/'&gt;
+base_url = 'https://swarajya-stg.corecotechnologies.com'
+employee_credentials = {'role': 'Employee', 'employee_id': '332', 'password': 'test@1234', 'auth_code': '111111', ...}
+    def test_back_button_after_logout_TC_LOGIN_035(self, page, base_url, employee_credentials):
+        """Browser back after logout should not expose cached dashboard."""
+        </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(login): enable direct python3 execution, auto-venv, and pytest compatibility
</commit_message>
<xml_diff>
--- a/test_data/login_test_cases.xlsx
+++ b/test_data/login_test_cases.xlsx
@@ -529,7 +529,7 @@
       </c>
       <c r="L2" s="0" t="inlineStr">
         <is>
-          <t>2026-08-28 20:21:39</t>
+          <t>2026-09-03 11:51:32</t>
         </is>
       </c>
       <c r="M2" s="0" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="L4" s="0" t="inlineStr">
         <is>
-          <t>2026-08-28 20:21:41</t>
+          <t>2026-09-03 11:12:38</t>
         </is>
       </c>
       <c r="M4" s="0" t="inlineStr">
@@ -2242,7 +2242,7 @@
       </c>
       <c r="L2" s="0" t="inlineStr">
         <is>
-          <t>2026-08-28 20:21:41</t>
+          <t>2026-09-03 11:12:39</t>
         </is>
       </c>
       <c r="M2" s="0" t="inlineStr">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="L3" s="0" t="inlineStr">
         <is>
-          <t>2026-08-28 20:21:42</t>
+          <t>2026-09-03 11:12:40</t>
         </is>
       </c>
       <c r="M3" s="0" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="L6" s="0" t="inlineStr">
         <is>
-          <t>2026-08-28 20:21:42</t>
+          <t>2026-09-03 11:12:40</t>
         </is>
       </c>
       <c r="M6" s="0" t="inlineStr">
@@ -2542,7 +2542,7 @@
       </c>
       <c r="L7" s="0" t="inlineStr">
         <is>
-          <t>2026-08-28 20:21:43</t>
+          <t>2026-09-03 11:12:41</t>
         </is>
       </c>
       <c r="M7" s="0" t="inlineStr">

</xml_diff>

<commit_message>
feat: consolidate direct execution, auto-venv, VS Code debug configurations, and stability fixes across all modules
</commit_message>
<xml_diff>
--- a/test_data/login_test_cases.xlsx
+++ b/test_data/login_test_cases.xlsx
@@ -529,7 +529,7 @@
       </c>
       <c r="L2" s="0" t="inlineStr">
         <is>
-          <t>2026-08-28 20:21:39</t>
+          <t>2026-09-03 11:51:32</t>
         </is>
       </c>
       <c r="M2" s="0" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="L4" s="0" t="inlineStr">
         <is>
-          <t>2026-08-28 20:21:41</t>
+          <t>2026-09-03 11:12:38</t>
         </is>
       </c>
       <c r="M4" s="0" t="inlineStr">
@@ -2242,7 +2242,7 @@
       </c>
       <c r="L2" s="0" t="inlineStr">
         <is>
-          <t>2026-08-28 20:21:41</t>
+          <t>2026-09-03 11:12:39</t>
         </is>
       </c>
       <c r="M2" s="0" t="inlineStr">
@@ -2308,7 +2308,7 @@
       </c>
       <c r="L3" s="0" t="inlineStr">
         <is>
-          <t>2026-08-28 20:21:42</t>
+          <t>2026-09-03 11:12:40</t>
         </is>
       </c>
       <c r="M3" s="0" t="inlineStr">
@@ -2476,7 +2476,7 @@
       </c>
       <c r="L6" s="0" t="inlineStr">
         <is>
-          <t>2026-08-28 20:21:42</t>
+          <t>2026-09-03 11:12:40</t>
         </is>
       </c>
       <c r="M6" s="0" t="inlineStr">
@@ -2542,7 +2542,7 @@
       </c>
       <c r="L7" s="0" t="inlineStr">
         <is>
-          <t>2026-08-28 20:21:43</t>
+          <t>2026-09-03 11:12:41</t>
         </is>
       </c>
       <c r="M7" s="0" t="inlineStr">

</xml_diff>